<commit_message>
feat: root-cause tagging with SQL rules and Claude (#8)
</commit_message>
<xml_diff>
--- a/audit/audit_sheet.xlsx
+++ b/audit/audit_sheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sampath.sho\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E409A488-678B-456C-BF02-65B6B517D096}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{832C1788-B15B-46EE-8D1C-0A3A97EACF54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="22780" windowHeight="14540" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2356" uniqueCount="1079">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4646" uniqueCount="1082">
   <si>
     <t>recall_number</t>
   </si>
@@ -3242,9 +3242,6 @@
     <t xml:space="preserve">	ranitidine hydrochloride</t>
   </si>
   <si>
-    <t>Zantac = ranitidine, NDMA</t>
-  </si>
-  <si>
     <t>epinephrine bitartrate + lidocaine hydrochloride + tetracaine hydrochloride</t>
   </si>
   <si>
@@ -3258,13 +3255,35 @@
   </si>
   <si>
     <t>hyphen joins the drugs; insanitary conditions</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Zantac = ranitidine, NDMA, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>Relabeled from CGMP on Oct 13 after re-checking the audit rules.</t>
+    </r>
+  </si>
+  <si>
+    <t>Relabeled from CGMP on Oct 13 after re-checking the audit rules.</t>
+  </si>
+  <si>
+    <t>zip code in leftovers, Relabeled from CGMP on Oct 13 after re-checking the audit rules.</t>
+  </si>
+  <si>
+    <t>Relabeled from Chemical or foreign contamination on Oct 13 after re-checking the audit rules.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -3280,6 +3299,11 @@
       <b/>
       <sz val="10"/>
       <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="4">
@@ -3312,7 +3336,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -3327,6 +3351,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -4364,9 +4391,11 @@
         <v>25</v>
       </c>
       <c r="Q15" s="4" t="s">
-        <v>1017</v>
-      </c>
-      <c r="R15" s="4"/>
+        <v>1027</v>
+      </c>
+      <c r="R15" s="6" t="s">
+        <v>1081</v>
+      </c>
     </row>
     <row r="16" spans="1:18" ht="50" x14ac:dyDescent="0.35">
       <c r="A16" s="3" t="s">
@@ -6114,9 +6143,11 @@
         <v>25</v>
       </c>
       <c r="Q52" s="4" t="s">
-        <v>1012</v>
-      </c>
-      <c r="R52" s="4"/>
+        <v>1025</v>
+      </c>
+      <c r="R52" s="6" t="s">
+        <v>1079</v>
+      </c>
     </row>
     <row r="53" spans="1:18" ht="50" x14ac:dyDescent="0.35">
       <c r="A53" s="3" t="s">
@@ -6526,7 +6557,7 @@
       </c>
       <c r="R61" s="4"/>
     </row>
-    <row r="62" spans="1:18" ht="25" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:18" ht="37.5" x14ac:dyDescent="0.35">
       <c r="A62" s="3" t="s">
         <v>367</v>
       </c>
@@ -6566,13 +6597,13 @@
         <v>25</v>
       </c>
       <c r="Q62" s="4" t="s">
-        <v>1012</v>
-      </c>
-      <c r="R62" s="4" t="s">
-        <v>1052</v>
-      </c>
-    </row>
-    <row r="63" spans="1:18" ht="25" x14ac:dyDescent="0.35">
+        <v>1031</v>
+      </c>
+      <c r="R62" s="6" t="s">
+        <v>1080</v>
+      </c>
+    </row>
+    <row r="63" spans="1:18" ht="37.5" x14ac:dyDescent="0.35">
       <c r="A63" s="3" t="s">
         <v>373</v>
       </c>
@@ -6612,10 +6643,10 @@
         <v>25</v>
       </c>
       <c r="Q63" s="4" t="s">
-        <v>1012</v>
-      </c>
-      <c r="R63" s="4" t="s">
-        <v>1052</v>
+        <v>1031</v>
+      </c>
+      <c r="R63" s="6" t="s">
+        <v>1080</v>
       </c>
     </row>
     <row r="64" spans="1:18" ht="50" x14ac:dyDescent="0.35">
@@ -6848,10 +6879,10 @@
         <v>25</v>
       </c>
       <c r="Q68" s="4" t="s">
-        <v>1012</v>
-      </c>
-      <c r="R68" s="4" t="s">
-        <v>1073</v>
+        <v>1021</v>
+      </c>
+      <c r="R68" s="6" t="s">
+        <v>1078</v>
       </c>
     </row>
     <row r="69" spans="1:18" ht="75" x14ac:dyDescent="0.35">
@@ -6887,7 +6918,7 @@
         <v>1043</v>
       </c>
       <c r="N69" s="4" t="s">
-        <v>1074</v>
+        <v>1073</v>
       </c>
       <c r="O69" s="4" t="s">
         <v>26</v>
@@ -6899,7 +6930,7 @@
         <v>497</v>
       </c>
       <c r="R69" s="4" t="s">
-        <v>1075</v>
+        <v>1074</v>
       </c>
     </row>
     <row r="70" spans="1:18" ht="25" x14ac:dyDescent="0.35">
@@ -6988,9 +7019,11 @@
         <v>25</v>
       </c>
       <c r="Q71" s="4" t="s">
-        <v>1012</v>
-      </c>
-      <c r="R71" s="4"/>
+        <v>1021</v>
+      </c>
+      <c r="R71" s="6" t="s">
+        <v>1079</v>
+      </c>
     </row>
     <row r="72" spans="1:18" ht="25" x14ac:dyDescent="0.35">
       <c r="A72" s="3" t="s">
@@ -7080,9 +7113,11 @@
         <v>25</v>
       </c>
       <c r="Q73" s="4" t="s">
-        <v>1012</v>
-      </c>
-      <c r="R73" s="4"/>
+        <v>497</v>
+      </c>
+      <c r="R73" s="6" t="s">
+        <v>1079</v>
+      </c>
     </row>
     <row r="74" spans="1:18" ht="37.5" x14ac:dyDescent="0.35">
       <c r="A74" s="3" t="s">
@@ -7393,7 +7428,7 @@
         <v>1043</v>
       </c>
       <c r="N80" s="4" t="s">
-        <v>1076</v>
+        <v>1075</v>
       </c>
       <c r="O80" s="4" t="s">
         <v>95</v>
@@ -7483,7 +7518,7 @@
         <v>1043</v>
       </c>
       <c r="N82" s="4" t="s">
-        <v>1077</v>
+        <v>1076</v>
       </c>
       <c r="O82" s="4" t="s">
         <v>95</v>
@@ -7495,7 +7530,7 @@
         <v>1012</v>
       </c>
       <c r="R82" s="4" t="s">
-        <v>1078</v>
+        <v>1077</v>
       </c>
     </row>
     <row r="83" spans="1:18" ht="37.5" x14ac:dyDescent="0.35">
@@ -7529,7 +7564,7 @@
         <v>1043</v>
       </c>
       <c r="N83" s="4" t="s">
-        <v>1077</v>
+        <v>1076</v>
       </c>
       <c r="O83" s="4" t="s">
         <v>95</v>
@@ -7541,7 +7576,7 @@
         <v>1012</v>
       </c>
       <c r="R83" s="4" t="s">
-        <v>1078</v>
+        <v>1077</v>
       </c>
     </row>
     <row r="84" spans="1:18" ht="37.5" x14ac:dyDescent="0.35">
@@ -7732,9 +7767,11 @@
         <v>25</v>
       </c>
       <c r="Q87" s="4" t="s">
-        <v>1012</v>
-      </c>
-      <c r="R87" s="4"/>
+        <v>1021</v>
+      </c>
+      <c r="R87" s="6" t="s">
+        <v>1079</v>
+      </c>
     </row>
     <row r="88" spans="1:18" ht="37.5" x14ac:dyDescent="0.35">
       <c r="A88" s="3" t="s">
@@ -12246,6 +12283,7 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
feat: root-cause tagging with SQL rules and Claude (#8) (#25)
</commit_message>
<xml_diff>
--- a/audit/audit_sheet.xlsx
+++ b/audit/audit_sheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sampath.sho\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E409A488-678B-456C-BF02-65B6B517D096}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{832C1788-B15B-46EE-8D1C-0A3A97EACF54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="22780" windowHeight="14540" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2356" uniqueCount="1079">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4646" uniqueCount="1082">
   <si>
     <t>recall_number</t>
   </si>
@@ -3242,9 +3242,6 @@
     <t xml:space="preserve">	ranitidine hydrochloride</t>
   </si>
   <si>
-    <t>Zantac = ranitidine, NDMA</t>
-  </si>
-  <si>
     <t>epinephrine bitartrate + lidocaine hydrochloride + tetracaine hydrochloride</t>
   </si>
   <si>
@@ -3258,13 +3255,35 @@
   </si>
   <si>
     <t>hyphen joins the drugs; insanitary conditions</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Zantac = ranitidine, NDMA, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>Relabeled from CGMP on Oct 13 after re-checking the audit rules.</t>
+    </r>
+  </si>
+  <si>
+    <t>Relabeled from CGMP on Oct 13 after re-checking the audit rules.</t>
+  </si>
+  <si>
+    <t>zip code in leftovers, Relabeled from CGMP on Oct 13 after re-checking the audit rules.</t>
+  </si>
+  <si>
+    <t>Relabeled from Chemical or foreign contamination on Oct 13 after re-checking the audit rules.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -3280,6 +3299,11 @@
       <b/>
       <sz val="10"/>
       <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="4">
@@ -3312,7 +3336,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -3327,6 +3351,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -4364,9 +4391,11 @@
         <v>25</v>
       </c>
       <c r="Q15" s="4" t="s">
-        <v>1017</v>
-      </c>
-      <c r="R15" s="4"/>
+        <v>1027</v>
+      </c>
+      <c r="R15" s="6" t="s">
+        <v>1081</v>
+      </c>
     </row>
     <row r="16" spans="1:18" ht="50" x14ac:dyDescent="0.35">
       <c r="A16" s="3" t="s">
@@ -6114,9 +6143,11 @@
         <v>25</v>
       </c>
       <c r="Q52" s="4" t="s">
-        <v>1012</v>
-      </c>
-      <c r="R52" s="4"/>
+        <v>1025</v>
+      </c>
+      <c r="R52" s="6" t="s">
+        <v>1079</v>
+      </c>
     </row>
     <row r="53" spans="1:18" ht="50" x14ac:dyDescent="0.35">
       <c r="A53" s="3" t="s">
@@ -6526,7 +6557,7 @@
       </c>
       <c r="R61" s="4"/>
     </row>
-    <row r="62" spans="1:18" ht="25" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:18" ht="37.5" x14ac:dyDescent="0.35">
       <c r="A62" s="3" t="s">
         <v>367</v>
       </c>
@@ -6566,13 +6597,13 @@
         <v>25</v>
       </c>
       <c r="Q62" s="4" t="s">
-        <v>1012</v>
-      </c>
-      <c r="R62" s="4" t="s">
-        <v>1052</v>
-      </c>
-    </row>
-    <row r="63" spans="1:18" ht="25" x14ac:dyDescent="0.35">
+        <v>1031</v>
+      </c>
+      <c r="R62" s="6" t="s">
+        <v>1080</v>
+      </c>
+    </row>
+    <row r="63" spans="1:18" ht="37.5" x14ac:dyDescent="0.35">
       <c r="A63" s="3" t="s">
         <v>373</v>
       </c>
@@ -6612,10 +6643,10 @@
         <v>25</v>
       </c>
       <c r="Q63" s="4" t="s">
-        <v>1012</v>
-      </c>
-      <c r="R63" s="4" t="s">
-        <v>1052</v>
+        <v>1031</v>
+      </c>
+      <c r="R63" s="6" t="s">
+        <v>1080</v>
       </c>
     </row>
     <row r="64" spans="1:18" ht="50" x14ac:dyDescent="0.35">
@@ -6848,10 +6879,10 @@
         <v>25</v>
       </c>
       <c r="Q68" s="4" t="s">
-        <v>1012</v>
-      </c>
-      <c r="R68" s="4" t="s">
-        <v>1073</v>
+        <v>1021</v>
+      </c>
+      <c r="R68" s="6" t="s">
+        <v>1078</v>
       </c>
     </row>
     <row r="69" spans="1:18" ht="75" x14ac:dyDescent="0.35">
@@ -6887,7 +6918,7 @@
         <v>1043</v>
       </c>
       <c r="N69" s="4" t="s">
-        <v>1074</v>
+        <v>1073</v>
       </c>
       <c r="O69" s="4" t="s">
         <v>26</v>
@@ -6899,7 +6930,7 @@
         <v>497</v>
       </c>
       <c r="R69" s="4" t="s">
-        <v>1075</v>
+        <v>1074</v>
       </c>
     </row>
     <row r="70" spans="1:18" ht="25" x14ac:dyDescent="0.35">
@@ -6988,9 +7019,11 @@
         <v>25</v>
       </c>
       <c r="Q71" s="4" t="s">
-        <v>1012</v>
-      </c>
-      <c r="R71" s="4"/>
+        <v>1021</v>
+      </c>
+      <c r="R71" s="6" t="s">
+        <v>1079</v>
+      </c>
     </row>
     <row r="72" spans="1:18" ht="25" x14ac:dyDescent="0.35">
       <c r="A72" s="3" t="s">
@@ -7080,9 +7113,11 @@
         <v>25</v>
       </c>
       <c r="Q73" s="4" t="s">
-        <v>1012</v>
-      </c>
-      <c r="R73" s="4"/>
+        <v>497</v>
+      </c>
+      <c r="R73" s="6" t="s">
+        <v>1079</v>
+      </c>
     </row>
     <row r="74" spans="1:18" ht="37.5" x14ac:dyDescent="0.35">
       <c r="A74" s="3" t="s">
@@ -7393,7 +7428,7 @@
         <v>1043</v>
       </c>
       <c r="N80" s="4" t="s">
-        <v>1076</v>
+        <v>1075</v>
       </c>
       <c r="O80" s="4" t="s">
         <v>95</v>
@@ -7483,7 +7518,7 @@
         <v>1043</v>
       </c>
       <c r="N82" s="4" t="s">
-        <v>1077</v>
+        <v>1076</v>
       </c>
       <c r="O82" s="4" t="s">
         <v>95</v>
@@ -7495,7 +7530,7 @@
         <v>1012</v>
       </c>
       <c r="R82" s="4" t="s">
-        <v>1078</v>
+        <v>1077</v>
       </c>
     </row>
     <row r="83" spans="1:18" ht="37.5" x14ac:dyDescent="0.35">
@@ -7529,7 +7564,7 @@
         <v>1043</v>
       </c>
       <c r="N83" s="4" t="s">
-        <v>1077</v>
+        <v>1076</v>
       </c>
       <c r="O83" s="4" t="s">
         <v>95</v>
@@ -7541,7 +7576,7 @@
         <v>1012</v>
       </c>
       <c r="R83" s="4" t="s">
-        <v>1078</v>
+        <v>1077</v>
       </c>
     </row>
     <row r="84" spans="1:18" ht="37.5" x14ac:dyDescent="0.35">
@@ -7732,9 +7767,11 @@
         <v>25</v>
       </c>
       <c r="Q87" s="4" t="s">
-        <v>1012</v>
-      </c>
-      <c r="R87" s="4"/>
+        <v>1021</v>
+      </c>
+      <c r="R87" s="6" t="s">
+        <v>1079</v>
+      </c>
     </row>
     <row r="88" spans="1:18" ht="37.5" x14ac:dyDescent="0.35">
       <c r="A88" s="3" t="s">
@@ -12246,6 +12283,7 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
feat: Claude names drugs for recalls matching can't (#9)
</commit_message>
<xml_diff>
--- a/audit/audit_sheet.xlsx
+++ b/audit/audit_sheet.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sampath.sho\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{832C1788-B15B-46EE-8D1C-0A3A97EACF54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE6B71AC-06EF-4D20-B543-5C29DF5AB3AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="22780" windowHeight="14540" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4646" uniqueCount="1082">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2361" uniqueCount="1082">
   <si>
     <t>recall_number</t>
   </si>
@@ -3155,9 +3155,6 @@
     <t>no</t>
   </si>
   <si>
-    <t>evorphanol tartrate</t>
-  </si>
-  <si>
     <t>generic in brackets after the brand</t>
   </si>
   <si>
@@ -3246,9 +3243,6 @@
   </si>
   <si>
     <t>LET kit, actives only</t>
-  </si>
-  <si>
-    <t>prostaglandin</t>
   </si>
   <si>
     <t>papaverine + phentolamine</t>
@@ -3277,6 +3271,12 @@
   </si>
   <si>
     <t>Relabeled from Chemical or foreign contamination on Oct 13 after re-checking the audit rules.</t>
+  </si>
+  <si>
+    <t>levorphanol tartrate</t>
+  </si>
+  <si>
+    <t>papaverine + phentolamine + alprostadil</t>
   </si>
 </sst>
 </file>
@@ -3764,7 +3764,7 @@
         <v>1043</v>
       </c>
       <c r="N2" s="4" t="s">
-        <v>1044</v>
+        <v>1080</v>
       </c>
       <c r="O2" s="4" t="s">
         <v>26</v>
@@ -3776,7 +3776,7 @@
         <v>1027</v>
       </c>
       <c r="R2" s="4" t="s">
-        <v>1045</v>
+        <v>1044</v>
       </c>
     </row>
     <row r="3" spans="1:18" ht="37.5" x14ac:dyDescent="0.35">
@@ -4002,7 +4002,7 @@
         <v>1043</v>
       </c>
       <c r="N7" s="4" t="s">
-        <v>1046</v>
+        <v>1045</v>
       </c>
       <c r="O7" s="4" t="s">
         <v>95</v>
@@ -4014,7 +4014,7 @@
         <v>1014</v>
       </c>
       <c r="R7" s="4" t="s">
-        <v>1047</v>
+        <v>1046</v>
       </c>
     </row>
     <row r="8" spans="1:18" ht="62.5" x14ac:dyDescent="0.35">
@@ -4237,7 +4237,7 @@
       </c>
       <c r="L12" s="3"/>
       <c r="M12" s="4" t="s">
-        <v>1048</v>
+        <v>1047</v>
       </c>
       <c r="N12" s="4"/>
       <c r="O12" s="4" t="s">
@@ -4394,7 +4394,7 @@
         <v>1027</v>
       </c>
       <c r="R15" s="6" t="s">
-        <v>1081</v>
+        <v>1079</v>
       </c>
     </row>
     <row r="16" spans="1:18" ht="50" x14ac:dyDescent="0.35">
@@ -4430,7 +4430,7 @@
         <v>1043</v>
       </c>
       <c r="N16" s="4" t="s">
-        <v>1049</v>
+        <v>1048</v>
       </c>
       <c r="O16" s="4" t="s">
         <v>26</v>
@@ -4810,7 +4810,7 @@
         <v>1043</v>
       </c>
       <c r="N24" s="4" t="s">
-        <v>1050</v>
+        <v>1049</v>
       </c>
       <c r="O24" s="4" t="s">
         <v>26</v>
@@ -4902,7 +4902,7 @@
         <v>1043</v>
       </c>
       <c r="N26" s="4" t="s">
-        <v>1051</v>
+        <v>1050</v>
       </c>
       <c r="O26" s="4" t="s">
         <v>95</v>
@@ -4945,7 +4945,7 @@
       </c>
       <c r="L27" s="3"/>
       <c r="M27" s="4" t="s">
-        <v>1048</v>
+        <v>1047</v>
       </c>
       <c r="N27" s="4"/>
       <c r="O27" s="4" t="s">
@@ -4958,7 +4958,7 @@
         <v>497</v>
       </c>
       <c r="R27" s="4" t="s">
-        <v>1052</v>
+        <v>1051</v>
       </c>
     </row>
     <row r="28" spans="1:18" ht="37.5" x14ac:dyDescent="0.35">
@@ -5085,7 +5085,7 @@
       </c>
       <c r="L30" s="3"/>
       <c r="M30" s="4" t="s">
-        <v>1048</v>
+        <v>1047</v>
       </c>
       <c r="N30" s="4"/>
       <c r="O30" s="4" t="s">
@@ -5127,7 +5127,7 @@
       </c>
       <c r="L31" s="3"/>
       <c r="M31" s="4" t="s">
-        <v>1048</v>
+        <v>1047</v>
       </c>
       <c r="N31" s="4"/>
       <c r="O31" s="4" t="s">
@@ -5226,7 +5226,7 @@
         <v>1043</v>
       </c>
       <c r="N33" s="4" t="s">
-        <v>1053</v>
+        <v>1052</v>
       </c>
       <c r="O33" s="4" t="s">
         <v>26</v>
@@ -5238,7 +5238,7 @@
         <v>1014</v>
       </c>
       <c r="R33" s="4" t="s">
-        <v>1054</v>
+        <v>1053</v>
       </c>
     </row>
     <row r="34" spans="1:18" ht="62.5" x14ac:dyDescent="0.35">
@@ -5320,7 +5320,7 @@
         <v>1043</v>
       </c>
       <c r="N35" s="4" t="s">
-        <v>1055</v>
+        <v>1054</v>
       </c>
       <c r="O35" s="4" t="s">
         <v>95</v>
@@ -5332,7 +5332,7 @@
         <v>1014</v>
       </c>
       <c r="R35" s="4" t="s">
-        <v>1056</v>
+        <v>1055</v>
       </c>
     </row>
     <row r="36" spans="1:18" ht="37.5" x14ac:dyDescent="0.35">
@@ -5512,7 +5512,7 @@
         <v>1043</v>
       </c>
       <c r="N39" s="4" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
       <c r="O39" s="4" t="s">
         <v>26</v>
@@ -5524,7 +5524,7 @@
         <v>1014</v>
       </c>
       <c r="R39" s="4" t="s">
-        <v>1058</v>
+        <v>1057</v>
       </c>
     </row>
     <row r="40" spans="1:18" ht="37.5" x14ac:dyDescent="0.35">
@@ -5564,7 +5564,7 @@
         <v>1043</v>
       </c>
       <c r="N40" s="4" t="s">
-        <v>1059</v>
+        <v>1058</v>
       </c>
       <c r="O40" s="4" t="s">
         <v>26</v>
@@ -5576,7 +5576,7 @@
         <v>1012</v>
       </c>
       <c r="R40" s="4" t="s">
-        <v>1060</v>
+        <v>1059</v>
       </c>
     </row>
     <row r="41" spans="1:18" ht="37.5" x14ac:dyDescent="0.35">
@@ -5612,7 +5612,7 @@
         <v>1043</v>
       </c>
       <c r="N41" s="4" t="s">
-        <v>1061</v>
+        <v>1060</v>
       </c>
       <c r="O41" s="4" t="s">
         <v>26</v>
@@ -5624,7 +5624,7 @@
         <v>1012</v>
       </c>
       <c r="R41" s="4" t="s">
-        <v>1062</v>
+        <v>1061</v>
       </c>
     </row>
     <row r="42" spans="1:18" ht="50" x14ac:dyDescent="0.35">
@@ -5800,7 +5800,7 @@
         <v>1043</v>
       </c>
       <c r="N45" s="4" t="s">
-        <v>1063</v>
+        <v>1062</v>
       </c>
       <c r="O45" s="4" t="s">
         <v>95</v>
@@ -5892,7 +5892,7 @@
         <v>1043</v>
       </c>
       <c r="N47" s="4" t="s">
-        <v>1061</v>
+        <v>1060</v>
       </c>
       <c r="O47" s="4" t="s">
         <v>95</v>
@@ -5904,7 +5904,7 @@
         <v>1014</v>
       </c>
       <c r="R47" s="4" t="s">
-        <v>1064</v>
+        <v>1063</v>
       </c>
     </row>
     <row r="48" spans="1:18" ht="62.5" x14ac:dyDescent="0.35">
@@ -6146,7 +6146,7 @@
         <v>1025</v>
       </c>
       <c r="R52" s="6" t="s">
-        <v>1079</v>
+        <v>1077</v>
       </c>
     </row>
     <row r="53" spans="1:18" ht="50" x14ac:dyDescent="0.35">
@@ -6358,7 +6358,7 @@
         <v>1043</v>
       </c>
       <c r="N57" s="4" t="s">
-        <v>1065</v>
+        <v>1064</v>
       </c>
       <c r="O57" s="4" t="s">
         <v>95</v>
@@ -6404,7 +6404,7 @@
         <v>1043</v>
       </c>
       <c r="N58" s="4" t="s">
-        <v>1066</v>
+        <v>1065</v>
       </c>
       <c r="O58" s="4" t="s">
         <v>26</v>
@@ -6416,7 +6416,7 @@
         <v>1012</v>
       </c>
       <c r="R58" s="4" t="s">
-        <v>1067</v>
+        <v>1066</v>
       </c>
     </row>
     <row r="59" spans="1:18" ht="75" x14ac:dyDescent="0.35">
@@ -6452,7 +6452,7 @@
         <v>1043</v>
       </c>
       <c r="N59" s="4" t="s">
-        <v>1066</v>
+        <v>1065</v>
       </c>
       <c r="O59" s="4" t="s">
         <v>26</v>
@@ -6464,7 +6464,7 @@
         <v>1012</v>
       </c>
       <c r="R59" s="4" t="s">
-        <v>1067</v>
+        <v>1066</v>
       </c>
     </row>
     <row r="60" spans="1:18" ht="25" x14ac:dyDescent="0.35">
@@ -6495,7 +6495,7 @@
       </c>
       <c r="L60" s="3"/>
       <c r="M60" s="4" t="s">
-        <v>1048</v>
+        <v>1047</v>
       </c>
       <c r="N60" s="4"/>
       <c r="O60" s="4" t="s">
@@ -6587,7 +6587,7 @@
       </c>
       <c r="L62" s="3"/>
       <c r="M62" s="4" t="s">
-        <v>1048</v>
+        <v>1047</v>
       </c>
       <c r="N62" s="4"/>
       <c r="O62" s="4" t="s">
@@ -6600,7 +6600,7 @@
         <v>1031</v>
       </c>
       <c r="R62" s="6" t="s">
-        <v>1080</v>
+        <v>1078</v>
       </c>
     </row>
     <row r="63" spans="1:18" ht="37.5" x14ac:dyDescent="0.35">
@@ -6633,7 +6633,7 @@
       </c>
       <c r="L63" s="3"/>
       <c r="M63" s="4" t="s">
-        <v>1048</v>
+        <v>1047</v>
       </c>
       <c r="N63" s="4"/>
       <c r="O63" s="4" t="s">
@@ -6646,7 +6646,7 @@
         <v>1031</v>
       </c>
       <c r="R63" s="6" t="s">
-        <v>1080</v>
+        <v>1078</v>
       </c>
     </row>
     <row r="64" spans="1:18" ht="50" x14ac:dyDescent="0.35">
@@ -6682,7 +6682,7 @@
         <v>1043</v>
       </c>
       <c r="N64" s="4" t="s">
-        <v>1068</v>
+        <v>1067</v>
       </c>
       <c r="O64" s="4" t="s">
         <v>26</v>
@@ -6694,7 +6694,7 @@
         <v>1014</v>
       </c>
       <c r="R64" s="4" t="s">
-        <v>1069</v>
+        <v>1068</v>
       </c>
     </row>
     <row r="65" spans="1:18" ht="25" x14ac:dyDescent="0.35">
@@ -6725,7 +6725,7 @@
       </c>
       <c r="L65" s="3"/>
       <c r="M65" s="4" t="s">
-        <v>1048</v>
+        <v>1047</v>
       </c>
       <c r="N65" s="4"/>
       <c r="O65" s="4" t="s">
@@ -6774,7 +6774,7 @@
         <v>1043</v>
       </c>
       <c r="N66" s="4" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="O66" s="4" t="s">
         <v>95</v>
@@ -6786,7 +6786,7 @@
         <v>1014</v>
       </c>
       <c r="R66" s="4" t="s">
-        <v>1071</v>
+        <v>1070</v>
       </c>
     </row>
     <row r="67" spans="1:18" ht="37.5" x14ac:dyDescent="0.35">
@@ -6872,7 +6872,7 @@
         <v>26</v>
       </c>
       <c r="N68" s="4" t="s">
-        <v>1072</v>
+        <v>1071</v>
       </c>
       <c r="O68" s="4"/>
       <c r="P68" s="4" t="s">
@@ -6882,7 +6882,7 @@
         <v>1021</v>
       </c>
       <c r="R68" s="6" t="s">
-        <v>1078</v>
+        <v>1076</v>
       </c>
     </row>
     <row r="69" spans="1:18" ht="75" x14ac:dyDescent="0.35">
@@ -6918,7 +6918,7 @@
         <v>1043</v>
       </c>
       <c r="N69" s="4" t="s">
-        <v>1073</v>
+        <v>1072</v>
       </c>
       <c r="O69" s="4" t="s">
         <v>26</v>
@@ -6930,7 +6930,7 @@
         <v>497</v>
       </c>
       <c r="R69" s="4" t="s">
-        <v>1074</v>
+        <v>1073</v>
       </c>
     </row>
     <row r="70" spans="1:18" ht="25" x14ac:dyDescent="0.35">
@@ -6961,7 +6961,7 @@
       </c>
       <c r="L70" s="3"/>
       <c r="M70" s="4" t="s">
-        <v>1048</v>
+        <v>1047</v>
       </c>
       <c r="N70" s="4"/>
       <c r="O70" s="4" t="s">
@@ -7022,7 +7022,7 @@
         <v>1021</v>
       </c>
       <c r="R71" s="6" t="s">
-        <v>1079</v>
+        <v>1077</v>
       </c>
     </row>
     <row r="72" spans="1:18" ht="25" x14ac:dyDescent="0.35">
@@ -7072,7 +7072,7 @@
         <v>1014</v>
       </c>
       <c r="R72" s="4" t="s">
-        <v>1052</v>
+        <v>1051</v>
       </c>
     </row>
     <row r="73" spans="1:18" ht="37.5" x14ac:dyDescent="0.35">
@@ -7103,7 +7103,7 @@
       </c>
       <c r="L73" s="3"/>
       <c r="M73" s="4" t="s">
-        <v>1048</v>
+        <v>1047</v>
       </c>
       <c r="N73" s="4"/>
       <c r="O73" s="4" t="s">
@@ -7116,7 +7116,7 @@
         <v>497</v>
       </c>
       <c r="R73" s="6" t="s">
-        <v>1079</v>
+        <v>1077</v>
       </c>
     </row>
     <row r="74" spans="1:18" ht="37.5" x14ac:dyDescent="0.35">
@@ -7245,7 +7245,7 @@
       </c>
       <c r="L76" s="3"/>
       <c r="M76" s="4" t="s">
-        <v>1048</v>
+        <v>1047</v>
       </c>
       <c r="N76" s="4"/>
       <c r="O76" s="4" t="s">
@@ -7258,7 +7258,7 @@
         <v>1012</v>
       </c>
       <c r="R76" s="4" t="s">
-        <v>1052</v>
+        <v>1051</v>
       </c>
     </row>
     <row r="77" spans="1:18" ht="37.5" x14ac:dyDescent="0.35">
@@ -7292,7 +7292,7 @@
         <v>1043</v>
       </c>
       <c r="N77" s="4" t="s">
-        <v>1065</v>
+        <v>1064</v>
       </c>
       <c r="O77" s="4" t="s">
         <v>95</v>
@@ -7336,7 +7336,7 @@
         <v>1043</v>
       </c>
       <c r="N78" s="4" t="s">
-        <v>1065</v>
+        <v>1064</v>
       </c>
       <c r="O78" s="4" t="s">
         <v>95</v>
@@ -7428,7 +7428,7 @@
         <v>1043</v>
       </c>
       <c r="N80" s="4" t="s">
-        <v>1075</v>
+        <v>758</v>
       </c>
       <c r="O80" s="4" t="s">
         <v>95</v>
@@ -7518,7 +7518,7 @@
         <v>1043</v>
       </c>
       <c r="N82" s="4" t="s">
-        <v>1076</v>
+        <v>1074</v>
       </c>
       <c r="O82" s="4" t="s">
         <v>95</v>
@@ -7530,7 +7530,7 @@
         <v>1012</v>
       </c>
       <c r="R82" s="4" t="s">
-        <v>1077</v>
+        <v>1075</v>
       </c>
     </row>
     <row r="83" spans="1:18" ht="37.5" x14ac:dyDescent="0.35">
@@ -7564,7 +7564,7 @@
         <v>1043</v>
       </c>
       <c r="N83" s="4" t="s">
-        <v>1076</v>
+        <v>1081</v>
       </c>
       <c r="O83" s="4" t="s">
         <v>95</v>
@@ -7576,7 +7576,7 @@
         <v>1012</v>
       </c>
       <c r="R83" s="4" t="s">
-        <v>1077</v>
+        <v>1075</v>
       </c>
     </row>
     <row r="84" spans="1:18" ht="37.5" x14ac:dyDescent="0.35">
@@ -7770,7 +7770,7 @@
         <v>1021</v>
       </c>
       <c r="R87" s="6" t="s">
-        <v>1079</v>
+        <v>1077</v>
       </c>
     </row>
     <row r="88" spans="1:18" ht="37.5" x14ac:dyDescent="0.35">
@@ -7849,7 +7849,7 @@
       </c>
       <c r="L89" s="3"/>
       <c r="M89" s="4" t="s">
-        <v>1048</v>
+        <v>1047</v>
       </c>
       <c r="N89" s="4"/>
       <c r="O89" s="4" t="s">
@@ -7893,7 +7893,7 @@
       </c>
       <c r="L90" s="3"/>
       <c r="M90" s="4" t="s">
-        <v>1048</v>
+        <v>1047</v>
       </c>
       <c r="N90" s="4"/>
       <c r="O90" s="4" t="s">
@@ -7937,7 +7937,7 @@
       </c>
       <c r="L91" s="3"/>
       <c r="M91" s="4" t="s">
-        <v>1048</v>
+        <v>1047</v>
       </c>
       <c r="N91" s="4"/>
       <c r="O91" s="4" t="s">
@@ -7981,7 +7981,7 @@
       </c>
       <c r="L92" s="3"/>
       <c r="M92" s="4" t="s">
-        <v>1048</v>
+        <v>1047</v>
       </c>
       <c r="N92" s="4"/>
       <c r="O92" s="4" t="s">
@@ -8025,7 +8025,7 @@
       </c>
       <c r="L93" s="3"/>
       <c r="M93" s="4" t="s">
-        <v>1048</v>
+        <v>1047</v>
       </c>
       <c r="N93" s="4"/>
       <c r="O93" s="4" t="s">
@@ -8069,7 +8069,7 @@
       </c>
       <c r="L94" s="3"/>
       <c r="M94" s="4" t="s">
-        <v>1048</v>
+        <v>1047</v>
       </c>
       <c r="N94" s="4"/>
       <c r="O94" s="4" t="s">
@@ -8113,7 +8113,7 @@
       </c>
       <c r="L95" s="3"/>
       <c r="M95" s="4" t="s">
-        <v>1048</v>
+        <v>1047</v>
       </c>
       <c r="N95" s="4"/>
       <c r="O95" s="4" t="s">
@@ -8155,7 +8155,7 @@
       </c>
       <c r="L96" s="3"/>
       <c r="M96" s="4" t="s">
-        <v>1048</v>
+        <v>1047</v>
       </c>
       <c r="N96" s="4"/>
       <c r="O96" s="4" t="s">
@@ -8197,7 +8197,7 @@
       </c>
       <c r="L97" s="3"/>
       <c r="M97" s="4" t="s">
-        <v>1048</v>
+        <v>1047</v>
       </c>
       <c r="N97" s="4"/>
       <c r="O97" s="4" t="s">
@@ -8333,7 +8333,7 @@
       </c>
       <c r="L100" s="3"/>
       <c r="M100" s="4" t="s">
-        <v>1048</v>
+        <v>1047</v>
       </c>
       <c r="N100" s="4"/>
       <c r="O100" s="4" t="s">
@@ -8381,7 +8381,7 @@
       </c>
       <c r="L101" s="3"/>
       <c r="M101" s="4" t="s">
-        <v>1048</v>
+        <v>1047</v>
       </c>
       <c r="N101" s="4"/>
       <c r="O101" s="4" t="s">

</xml_diff>

<commit_message>
feat: Claude names drugs for recalls matching can't (#9) (#27)
</commit_message>
<xml_diff>
--- a/audit/audit_sheet.xlsx
+++ b/audit/audit_sheet.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sampath.sho\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{832C1788-B15B-46EE-8D1C-0A3A97EACF54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE6B71AC-06EF-4D20-B543-5C29DF5AB3AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="22780" windowHeight="14540" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4646" uniqueCount="1082">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2361" uniqueCount="1082">
   <si>
     <t>recall_number</t>
   </si>
@@ -3155,9 +3155,6 @@
     <t>no</t>
   </si>
   <si>
-    <t>evorphanol tartrate</t>
-  </si>
-  <si>
     <t>generic in brackets after the brand</t>
   </si>
   <si>
@@ -3246,9 +3243,6 @@
   </si>
   <si>
     <t>LET kit, actives only</t>
-  </si>
-  <si>
-    <t>prostaglandin</t>
   </si>
   <si>
     <t>papaverine + phentolamine</t>
@@ -3277,6 +3271,12 @@
   </si>
   <si>
     <t>Relabeled from Chemical or foreign contamination on Oct 13 after re-checking the audit rules.</t>
+  </si>
+  <si>
+    <t>levorphanol tartrate</t>
+  </si>
+  <si>
+    <t>papaverine + phentolamine + alprostadil</t>
   </si>
 </sst>
 </file>
@@ -3764,7 +3764,7 @@
         <v>1043</v>
       </c>
       <c r="N2" s="4" t="s">
-        <v>1044</v>
+        <v>1080</v>
       </c>
       <c r="O2" s="4" t="s">
         <v>26</v>
@@ -3776,7 +3776,7 @@
         <v>1027</v>
       </c>
       <c r="R2" s="4" t="s">
-        <v>1045</v>
+        <v>1044</v>
       </c>
     </row>
     <row r="3" spans="1:18" ht="37.5" x14ac:dyDescent="0.35">
@@ -4002,7 +4002,7 @@
         <v>1043</v>
       </c>
       <c r="N7" s="4" t="s">
-        <v>1046</v>
+        <v>1045</v>
       </c>
       <c r="O7" s="4" t="s">
         <v>95</v>
@@ -4014,7 +4014,7 @@
         <v>1014</v>
       </c>
       <c r="R7" s="4" t="s">
-        <v>1047</v>
+        <v>1046</v>
       </c>
     </row>
     <row r="8" spans="1:18" ht="62.5" x14ac:dyDescent="0.35">
@@ -4237,7 +4237,7 @@
       </c>
       <c r="L12" s="3"/>
       <c r="M12" s="4" t="s">
-        <v>1048</v>
+        <v>1047</v>
       </c>
       <c r="N12" s="4"/>
       <c r="O12" s="4" t="s">
@@ -4394,7 +4394,7 @@
         <v>1027</v>
       </c>
       <c r="R15" s="6" t="s">
-        <v>1081</v>
+        <v>1079</v>
       </c>
     </row>
     <row r="16" spans="1:18" ht="50" x14ac:dyDescent="0.35">
@@ -4430,7 +4430,7 @@
         <v>1043</v>
       </c>
       <c r="N16" s="4" t="s">
-        <v>1049</v>
+        <v>1048</v>
       </c>
       <c r="O16" s="4" t="s">
         <v>26</v>
@@ -4810,7 +4810,7 @@
         <v>1043</v>
       </c>
       <c r="N24" s="4" t="s">
-        <v>1050</v>
+        <v>1049</v>
       </c>
       <c r="O24" s="4" t="s">
         <v>26</v>
@@ -4902,7 +4902,7 @@
         <v>1043</v>
       </c>
       <c r="N26" s="4" t="s">
-        <v>1051</v>
+        <v>1050</v>
       </c>
       <c r="O26" s="4" t="s">
         <v>95</v>
@@ -4945,7 +4945,7 @@
       </c>
       <c r="L27" s="3"/>
       <c r="M27" s="4" t="s">
-        <v>1048</v>
+        <v>1047</v>
       </c>
       <c r="N27" s="4"/>
       <c r="O27" s="4" t="s">
@@ -4958,7 +4958,7 @@
         <v>497</v>
       </c>
       <c r="R27" s="4" t="s">
-        <v>1052</v>
+        <v>1051</v>
       </c>
     </row>
     <row r="28" spans="1:18" ht="37.5" x14ac:dyDescent="0.35">
@@ -5085,7 +5085,7 @@
       </c>
       <c r="L30" s="3"/>
       <c r="M30" s="4" t="s">
-        <v>1048</v>
+        <v>1047</v>
       </c>
       <c r="N30" s="4"/>
       <c r="O30" s="4" t="s">
@@ -5127,7 +5127,7 @@
       </c>
       <c r="L31" s="3"/>
       <c r="M31" s="4" t="s">
-        <v>1048</v>
+        <v>1047</v>
       </c>
       <c r="N31" s="4"/>
       <c r="O31" s="4" t="s">
@@ -5226,7 +5226,7 @@
         <v>1043</v>
       </c>
       <c r="N33" s="4" t="s">
-        <v>1053</v>
+        <v>1052</v>
       </c>
       <c r="O33" s="4" t="s">
         <v>26</v>
@@ -5238,7 +5238,7 @@
         <v>1014</v>
       </c>
       <c r="R33" s="4" t="s">
-        <v>1054</v>
+        <v>1053</v>
       </c>
     </row>
     <row r="34" spans="1:18" ht="62.5" x14ac:dyDescent="0.35">
@@ -5320,7 +5320,7 @@
         <v>1043</v>
       </c>
       <c r="N35" s="4" t="s">
-        <v>1055</v>
+        <v>1054</v>
       </c>
       <c r="O35" s="4" t="s">
         <v>95</v>
@@ -5332,7 +5332,7 @@
         <v>1014</v>
       </c>
       <c r="R35" s="4" t="s">
-        <v>1056</v>
+        <v>1055</v>
       </c>
     </row>
     <row r="36" spans="1:18" ht="37.5" x14ac:dyDescent="0.35">
@@ -5512,7 +5512,7 @@
         <v>1043</v>
       </c>
       <c r="N39" s="4" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
       <c r="O39" s="4" t="s">
         <v>26</v>
@@ -5524,7 +5524,7 @@
         <v>1014</v>
       </c>
       <c r="R39" s="4" t="s">
-        <v>1058</v>
+        <v>1057</v>
       </c>
     </row>
     <row r="40" spans="1:18" ht="37.5" x14ac:dyDescent="0.35">
@@ -5564,7 +5564,7 @@
         <v>1043</v>
       </c>
       <c r="N40" s="4" t="s">
-        <v>1059</v>
+        <v>1058</v>
       </c>
       <c r="O40" s="4" t="s">
         <v>26</v>
@@ -5576,7 +5576,7 @@
         <v>1012</v>
       </c>
       <c r="R40" s="4" t="s">
-        <v>1060</v>
+        <v>1059</v>
       </c>
     </row>
     <row r="41" spans="1:18" ht="37.5" x14ac:dyDescent="0.35">
@@ -5612,7 +5612,7 @@
         <v>1043</v>
       </c>
       <c r="N41" s="4" t="s">
-        <v>1061</v>
+        <v>1060</v>
       </c>
       <c r="O41" s="4" t="s">
         <v>26</v>
@@ -5624,7 +5624,7 @@
         <v>1012</v>
       </c>
       <c r="R41" s="4" t="s">
-        <v>1062</v>
+        <v>1061</v>
       </c>
     </row>
     <row r="42" spans="1:18" ht="50" x14ac:dyDescent="0.35">
@@ -5800,7 +5800,7 @@
         <v>1043</v>
       </c>
       <c r="N45" s="4" t="s">
-        <v>1063</v>
+        <v>1062</v>
       </c>
       <c r="O45" s="4" t="s">
         <v>95</v>
@@ -5892,7 +5892,7 @@
         <v>1043</v>
       </c>
       <c r="N47" s="4" t="s">
-        <v>1061</v>
+        <v>1060</v>
       </c>
       <c r="O47" s="4" t="s">
         <v>95</v>
@@ -5904,7 +5904,7 @@
         <v>1014</v>
       </c>
       <c r="R47" s="4" t="s">
-        <v>1064</v>
+        <v>1063</v>
       </c>
     </row>
     <row r="48" spans="1:18" ht="62.5" x14ac:dyDescent="0.35">
@@ -6146,7 +6146,7 @@
         <v>1025</v>
       </c>
       <c r="R52" s="6" t="s">
-        <v>1079</v>
+        <v>1077</v>
       </c>
     </row>
     <row r="53" spans="1:18" ht="50" x14ac:dyDescent="0.35">
@@ -6358,7 +6358,7 @@
         <v>1043</v>
       </c>
       <c r="N57" s="4" t="s">
-        <v>1065</v>
+        <v>1064</v>
       </c>
       <c r="O57" s="4" t="s">
         <v>95</v>
@@ -6404,7 +6404,7 @@
         <v>1043</v>
       </c>
       <c r="N58" s="4" t="s">
-        <v>1066</v>
+        <v>1065</v>
       </c>
       <c r="O58" s="4" t="s">
         <v>26</v>
@@ -6416,7 +6416,7 @@
         <v>1012</v>
       </c>
       <c r="R58" s="4" t="s">
-        <v>1067</v>
+        <v>1066</v>
       </c>
     </row>
     <row r="59" spans="1:18" ht="75" x14ac:dyDescent="0.35">
@@ -6452,7 +6452,7 @@
         <v>1043</v>
       </c>
       <c r="N59" s="4" t="s">
-        <v>1066</v>
+        <v>1065</v>
       </c>
       <c r="O59" s="4" t="s">
         <v>26</v>
@@ -6464,7 +6464,7 @@
         <v>1012</v>
       </c>
       <c r="R59" s="4" t="s">
-        <v>1067</v>
+        <v>1066</v>
       </c>
     </row>
     <row r="60" spans="1:18" ht="25" x14ac:dyDescent="0.35">
@@ -6495,7 +6495,7 @@
       </c>
       <c r="L60" s="3"/>
       <c r="M60" s="4" t="s">
-        <v>1048</v>
+        <v>1047</v>
       </c>
       <c r="N60" s="4"/>
       <c r="O60" s="4" t="s">
@@ -6587,7 +6587,7 @@
       </c>
       <c r="L62" s="3"/>
       <c r="M62" s="4" t="s">
-        <v>1048</v>
+        <v>1047</v>
       </c>
       <c r="N62" s="4"/>
       <c r="O62" s="4" t="s">
@@ -6600,7 +6600,7 @@
         <v>1031</v>
       </c>
       <c r="R62" s="6" t="s">
-        <v>1080</v>
+        <v>1078</v>
       </c>
     </row>
     <row r="63" spans="1:18" ht="37.5" x14ac:dyDescent="0.35">
@@ -6633,7 +6633,7 @@
       </c>
       <c r="L63" s="3"/>
       <c r="M63" s="4" t="s">
-        <v>1048</v>
+        <v>1047</v>
       </c>
       <c r="N63" s="4"/>
       <c r="O63" s="4" t="s">
@@ -6646,7 +6646,7 @@
         <v>1031</v>
       </c>
       <c r="R63" s="6" t="s">
-        <v>1080</v>
+        <v>1078</v>
       </c>
     </row>
     <row r="64" spans="1:18" ht="50" x14ac:dyDescent="0.35">
@@ -6682,7 +6682,7 @@
         <v>1043</v>
       </c>
       <c r="N64" s="4" t="s">
-        <v>1068</v>
+        <v>1067</v>
       </c>
       <c r="O64" s="4" t="s">
         <v>26</v>
@@ -6694,7 +6694,7 @@
         <v>1014</v>
       </c>
       <c r="R64" s="4" t="s">
-        <v>1069</v>
+        <v>1068</v>
       </c>
     </row>
     <row r="65" spans="1:18" ht="25" x14ac:dyDescent="0.35">
@@ -6725,7 +6725,7 @@
       </c>
       <c r="L65" s="3"/>
       <c r="M65" s="4" t="s">
-        <v>1048</v>
+        <v>1047</v>
       </c>
       <c r="N65" s="4"/>
       <c r="O65" s="4" t="s">
@@ -6774,7 +6774,7 @@
         <v>1043</v>
       </c>
       <c r="N66" s="4" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="O66" s="4" t="s">
         <v>95</v>
@@ -6786,7 +6786,7 @@
         <v>1014</v>
       </c>
       <c r="R66" s="4" t="s">
-        <v>1071</v>
+        <v>1070</v>
       </c>
     </row>
     <row r="67" spans="1:18" ht="37.5" x14ac:dyDescent="0.35">
@@ -6872,7 +6872,7 @@
         <v>26</v>
       </c>
       <c r="N68" s="4" t="s">
-        <v>1072</v>
+        <v>1071</v>
       </c>
       <c r="O68" s="4"/>
       <c r="P68" s="4" t="s">
@@ -6882,7 +6882,7 @@
         <v>1021</v>
       </c>
       <c r="R68" s="6" t="s">
-        <v>1078</v>
+        <v>1076</v>
       </c>
     </row>
     <row r="69" spans="1:18" ht="75" x14ac:dyDescent="0.35">
@@ -6918,7 +6918,7 @@
         <v>1043</v>
       </c>
       <c r="N69" s="4" t="s">
-        <v>1073</v>
+        <v>1072</v>
       </c>
       <c r="O69" s="4" t="s">
         <v>26</v>
@@ -6930,7 +6930,7 @@
         <v>497</v>
       </c>
       <c r="R69" s="4" t="s">
-        <v>1074</v>
+        <v>1073</v>
       </c>
     </row>
     <row r="70" spans="1:18" ht="25" x14ac:dyDescent="0.35">
@@ -6961,7 +6961,7 @@
       </c>
       <c r="L70" s="3"/>
       <c r="M70" s="4" t="s">
-        <v>1048</v>
+        <v>1047</v>
       </c>
       <c r="N70" s="4"/>
       <c r="O70" s="4" t="s">
@@ -7022,7 +7022,7 @@
         <v>1021</v>
       </c>
       <c r="R71" s="6" t="s">
-        <v>1079</v>
+        <v>1077</v>
       </c>
     </row>
     <row r="72" spans="1:18" ht="25" x14ac:dyDescent="0.35">
@@ -7072,7 +7072,7 @@
         <v>1014</v>
       </c>
       <c r="R72" s="4" t="s">
-        <v>1052</v>
+        <v>1051</v>
       </c>
     </row>
     <row r="73" spans="1:18" ht="37.5" x14ac:dyDescent="0.35">
@@ -7103,7 +7103,7 @@
       </c>
       <c r="L73" s="3"/>
       <c r="M73" s="4" t="s">
-        <v>1048</v>
+        <v>1047</v>
       </c>
       <c r="N73" s="4"/>
       <c r="O73" s="4" t="s">
@@ -7116,7 +7116,7 @@
         <v>497</v>
       </c>
       <c r="R73" s="6" t="s">
-        <v>1079</v>
+        <v>1077</v>
       </c>
     </row>
     <row r="74" spans="1:18" ht="37.5" x14ac:dyDescent="0.35">
@@ -7245,7 +7245,7 @@
       </c>
       <c r="L76" s="3"/>
       <c r="M76" s="4" t="s">
-        <v>1048</v>
+        <v>1047</v>
       </c>
       <c r="N76" s="4"/>
       <c r="O76" s="4" t="s">
@@ -7258,7 +7258,7 @@
         <v>1012</v>
       </c>
       <c r="R76" s="4" t="s">
-        <v>1052</v>
+        <v>1051</v>
       </c>
     </row>
     <row r="77" spans="1:18" ht="37.5" x14ac:dyDescent="0.35">
@@ -7292,7 +7292,7 @@
         <v>1043</v>
       </c>
       <c r="N77" s="4" t="s">
-        <v>1065</v>
+        <v>1064</v>
       </c>
       <c r="O77" s="4" t="s">
         <v>95</v>
@@ -7336,7 +7336,7 @@
         <v>1043</v>
       </c>
       <c r="N78" s="4" t="s">
-        <v>1065</v>
+        <v>1064</v>
       </c>
       <c r="O78" s="4" t="s">
         <v>95</v>
@@ -7428,7 +7428,7 @@
         <v>1043</v>
       </c>
       <c r="N80" s="4" t="s">
-        <v>1075</v>
+        <v>758</v>
       </c>
       <c r="O80" s="4" t="s">
         <v>95</v>
@@ -7518,7 +7518,7 @@
         <v>1043</v>
       </c>
       <c r="N82" s="4" t="s">
-        <v>1076</v>
+        <v>1074</v>
       </c>
       <c r="O82" s="4" t="s">
         <v>95</v>
@@ -7530,7 +7530,7 @@
         <v>1012</v>
       </c>
       <c r="R82" s="4" t="s">
-        <v>1077</v>
+        <v>1075</v>
       </c>
     </row>
     <row r="83" spans="1:18" ht="37.5" x14ac:dyDescent="0.35">
@@ -7564,7 +7564,7 @@
         <v>1043</v>
       </c>
       <c r="N83" s="4" t="s">
-        <v>1076</v>
+        <v>1081</v>
       </c>
       <c r="O83" s="4" t="s">
         <v>95</v>
@@ -7576,7 +7576,7 @@
         <v>1012</v>
       </c>
       <c r="R83" s="4" t="s">
-        <v>1077</v>
+        <v>1075</v>
       </c>
     </row>
     <row r="84" spans="1:18" ht="37.5" x14ac:dyDescent="0.35">
@@ -7770,7 +7770,7 @@
         <v>1021</v>
       </c>
       <c r="R87" s="6" t="s">
-        <v>1079</v>
+        <v>1077</v>
       </c>
     </row>
     <row r="88" spans="1:18" ht="37.5" x14ac:dyDescent="0.35">
@@ -7849,7 +7849,7 @@
       </c>
       <c r="L89" s="3"/>
       <c r="M89" s="4" t="s">
-        <v>1048</v>
+        <v>1047</v>
       </c>
       <c r="N89" s="4"/>
       <c r="O89" s="4" t="s">
@@ -7893,7 +7893,7 @@
       </c>
       <c r="L90" s="3"/>
       <c r="M90" s="4" t="s">
-        <v>1048</v>
+        <v>1047</v>
       </c>
       <c r="N90" s="4"/>
       <c r="O90" s="4" t="s">
@@ -7937,7 +7937,7 @@
       </c>
       <c r="L91" s="3"/>
       <c r="M91" s="4" t="s">
-        <v>1048</v>
+        <v>1047</v>
       </c>
       <c r="N91" s="4"/>
       <c r="O91" s="4" t="s">
@@ -7981,7 +7981,7 @@
       </c>
       <c r="L92" s="3"/>
       <c r="M92" s="4" t="s">
-        <v>1048</v>
+        <v>1047</v>
       </c>
       <c r="N92" s="4"/>
       <c r="O92" s="4" t="s">
@@ -8025,7 +8025,7 @@
       </c>
       <c r="L93" s="3"/>
       <c r="M93" s="4" t="s">
-        <v>1048</v>
+        <v>1047</v>
       </c>
       <c r="N93" s="4"/>
       <c r="O93" s="4" t="s">
@@ -8069,7 +8069,7 @@
       </c>
       <c r="L94" s="3"/>
       <c r="M94" s="4" t="s">
-        <v>1048</v>
+        <v>1047</v>
       </c>
       <c r="N94" s="4"/>
       <c r="O94" s="4" t="s">
@@ -8113,7 +8113,7 @@
       </c>
       <c r="L95" s="3"/>
       <c r="M95" s="4" t="s">
-        <v>1048</v>
+        <v>1047</v>
       </c>
       <c r="N95" s="4"/>
       <c r="O95" s="4" t="s">
@@ -8155,7 +8155,7 @@
       </c>
       <c r="L96" s="3"/>
       <c r="M96" s="4" t="s">
-        <v>1048</v>
+        <v>1047</v>
       </c>
       <c r="N96" s="4"/>
       <c r="O96" s="4" t="s">
@@ -8197,7 +8197,7 @@
       </c>
       <c r="L97" s="3"/>
       <c r="M97" s="4" t="s">
-        <v>1048</v>
+        <v>1047</v>
       </c>
       <c r="N97" s="4"/>
       <c r="O97" s="4" t="s">
@@ -8333,7 +8333,7 @@
       </c>
       <c r="L100" s="3"/>
       <c r="M100" s="4" t="s">
-        <v>1048</v>
+        <v>1047</v>
       </c>
       <c r="N100" s="4"/>
       <c r="O100" s="4" t="s">
@@ -8381,7 +8381,7 @@
       </c>
       <c r="L101" s="3"/>
       <c r="M101" s="4" t="s">
-        <v>1048</v>
+        <v>1047</v>
       </c>
       <c r="N101" s="4"/>
       <c r="O101" s="4" t="s">

</xml_diff>